<commit_message>
Update reports 2026-09-02 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-02.xlsx
+++ b/gex_pivot_levels_2026-09-02.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$9.12M</t>
+          <t>-$8.78M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$9.68M</t>
+          <t>+$9.33M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -577,12 +577,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$1.90M</t>
+          <t>-$1.83M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$1.98M</t>
+          <t>+$1.92M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$15.94M</t>
+          <t>-$16.26M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$17.45M</t>
+          <t>+$17.80M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$12.26M</t>
+          <t>-$12.49M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$17.75M</t>
+          <t>+$18.08M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-$4.78M</t>
+          <t>-$4.95M</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>+$10.91M</t>
+          <t>+$11.28M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -734,12 +734,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-$12.87M</t>
+          <t>-$13.28M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$14.95M</t>
+          <t>+$15.42M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>-$12.04M</t>
+          <t>-$12.40M</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>+$20.07M</t>
+          <t>+$20.66M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>-$9.84M</t>
+          <t>-$10.30M</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>+$22.55M</t>
+          <t>+$23.60M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -924,12 +924,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$3.23M</t>
+          <t>+$3.31M</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>+$24.61M</t>
+          <t>+$25.21M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$2.34M</t>
+          <t>+$2.31M</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$9.67M</t>
+          <t>+$9.52M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>+$21.30M</t>
+          <t>+$20.48M</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>+$27.79M</t>
+          <t>+$26.72M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1151,12 +1151,12 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>+$6.58M</t>
+          <t>+$6.28M</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>+$9.93M</t>
+          <t>+$9.48M</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1234,10 +1234,10 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>7736.28</v>
+        <v>7746.28</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>7725</v>
+        <v>7735</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
@@ -1246,12 +1246,12 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>+$3.09M</t>
+          <t>+$4.61M</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>+$4.23M</t>
+          <t>+$4.69M</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1261,37 +1261,8 @@
       </c>
       <c r="G24" s="6" t="inlineStr"/>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="n">
-        <v>7746.28</v>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>7735</v>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>+$4.61M</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>+$4.69M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3161,7 +3132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3273,12 +3244,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>+$21.30M</t>
+          <t>+$20.48M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>+$27.79M</t>
+          <t>+$26.72M</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3311,12 +3282,12 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>+$3.23M</t>
+          <t>+$3.31M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$24.61M</t>
+          <t>+$25.21M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3345,12 +3316,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>-$9.84M</t>
+          <t>-$10.30M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>+$22.55M</t>
+          <t>+$23.60M</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -3405,36 +3376,32 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7695.04</v>
+        <v>7611.28</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>767</v>
+        <v>7600</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>+$6.67M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-$12.40M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$20.12M</t>
+          <t>+$20.66M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3443,32 +3410,36 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>7611.28</v>
+        <v>7695.04</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>7600</v>
+        <v>767</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>-$12.04M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>+$6.67M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$20.07M</t>
+          <t>+$20.12M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -3477,36 +3448,32 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>7654.97</v>
+        <v>7596.28</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>763</v>
+        <v>7585</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-$13.04M</t>
+          <t>-$12.49M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>+$18.03M</t>
+          <t>+$18.08M</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -3515,104 +3482,108 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7596.28</v>
+        <v>7654.97</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>7585</v>
+        <v>763</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>-$13.04M</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>+$18.03M</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7591.28</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>7580</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>-$12.26M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>+$17.75M</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>-$16.26M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>+$17.80M</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B12" s="2" t="n">
         <v>7624.92</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C12" s="2" t="n">
         <v>760</v>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>-$12.20M</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>+$17.61M</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>7591.28</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>7580</v>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>-$15.94M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>+$17.45M</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3713,12 +3684,12 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>-$12.87M</t>
+          <t>-$13.28M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>+$14.95M</t>
+          <t>+$15.42M</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -3849,74 +3820,74 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>29427.92</v>
+        <v>7601.28</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>715</v>
+        <v>7590</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>-$2.88M</t>
+          <t>-$4.95M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>+$10.94M</t>
+          <t>+$11.28M</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>7601.28</v>
+        <v>29427.92</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>7590</v>
+        <v>715</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>-$4.78M</t>
+          <t>-$2.88M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>+$10.91M</t>
+          <t>+$10.94M</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -4039,104 +4010,104 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
+        <v>7676.28</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>7665</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>+$2.31M</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>+$9.52M</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
         <v>7711.28</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C25" s="5" t="n">
         <v>7700</v>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>+$6.58M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>+$9.93M</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$6.28M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$9.48M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B26" s="2" t="n">
         <v>7561.28</v>
       </c>
-      <c r="C25" s="2" t="n">
+      <c r="C26" s="2" t="n">
         <v>7550</v>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-$9.12M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$9.68M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$8.78M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$9.33M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>7676.28</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>7665</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$2.34M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$9.67M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4511,228 +4482,228 @@
       <c r="H36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>7736.28</v>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>7725</v>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>+$3.09M</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>+$4.23M</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr"/>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>28441.75</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>-$3.97M</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>+$3.98M</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>4271.3</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>-$3.18M</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>+$3.36M</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
-        <v>28441.75</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>691</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="B39" s="5" t="n">
+        <v>29181.38</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>709</v>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>-$3.97M</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>+$3.98M</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>4271.3</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>93</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-$3.18M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$3.36M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>-$1.04M</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>+$2.26M</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>7566.28</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>7555</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>-$1.83M</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>+$1.92M</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>4350.74</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>397</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>-$1.60M</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>+$1.90M</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n">
-        <v>29181.38</v>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>709</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="B42" s="5" t="n">
+        <v>29838.83</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>725</v>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>-$1.04M</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>+$2.26M</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>7566.28</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>7555</v>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>-$1.90M</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>+$1.98M</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>4350.74</v>
-      </c>
-      <c r="C42" s="2" t="n">
-        <v>397</v>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>-$1.60M</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>+$1.90M</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>+$1.70M</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>+$1.78M</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -4741,130 +4712,134 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>29838.83</v>
+        <v>28852.66</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>725</v>
+        <v>701</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>+$1.70M</t>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>-$993.19K</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>+$1.78M</t>
+          <t>+$1.64M</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>28852.66</v>
+        <v>4822.44</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>701</v>
+        <v>105</v>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>-$993.19K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>+$1.54M</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>+$1.64M</t>
+          <t>+$1.58M</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>4822.44</v>
+        <v>28770.48</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>105</v>
+        <v>699</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>+$1.54M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>-$914.24K</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>+$1.58M</t>
+          <t>+$1.06M</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>28770.48</v>
+        <v>4317.23</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>699</v>
+        <v>94</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>-$914.24K</t>
+          <t>-$572.12K</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>+$1.06M</t>
+          <t>+$1.00M</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -4879,178 +4854,174 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n">
-        <v>4317.23</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>94</v>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>-$572.12K</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>+$1.00M</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="B47" s="2" t="n">
+        <v>4383.62</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>-$873.43K</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>+$945.30K</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>88.26000000000001</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>+$729.67K</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>+$729.67K</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>4493.21</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>410</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>+$570.28K</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>+$698.57K</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>4383.62</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>-$873.43K</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>+$945.30K</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
-        <v>88.26000000000001</v>
-      </c>
-      <c r="C49" s="5" t="n">
-        <v>145</v>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="B50" s="5" t="n">
+        <v>94.34999999999999</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>155</v>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>+$729.67K</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>+$729.67K</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>+$475.62K</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>+$475.62K</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>4493.21</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>410</v>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>+$570.28K</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>+$698.57K</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>94.34999999999999</v>
+        <v>4438.41</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>155</v>
+        <v>405</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>+$475.62K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>-$134.19K</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>+$475.62K</t>
+          <t>+$355.48K</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -5061,38 +5032,42 @@
       <c r="H51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n">
-        <v>4438.41</v>
-      </c>
-      <c r="C52" s="5" t="n">
-        <v>405</v>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>-$134.19K</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>+$355.48K</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr"/>
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>29128.28</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>29080</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>-$165.74K</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>+$322.76K</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -5101,24 +5076,24 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>29128.28</v>
+        <v>29148.28</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>29080</v>
+        <v>29100</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>-$165.74K</t>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>+$61.06K</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>+$322.76K</t>
+          <t>+$287.86K</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -5128,43 +5103,43 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="n">
-        <v>29148.28</v>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>29100</v>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>+$61.06K</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>+$287.86K</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4361.7</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>398</v>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>-$238.03K</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>+$274.54K</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5173,40 +5148,36 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>4361.7</v>
+        <v>29048.28</v>
       </c>
       <c r="C55" s="5" t="n">
-        <v>398</v>
+        <v>29000</v>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>-$238.03K</t>
+          <t>-$52.92K</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>+$274.54K</t>
+          <t>+$272.74K</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -5215,10 +5186,10 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>29048.28</v>
+        <v>29098.28</v>
       </c>
       <c r="C56" s="5" t="n">
-        <v>29000</v>
+        <v>29050</v>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
@@ -5227,12 +5198,12 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>-$52.92K</t>
+          <t>-$52.34K</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>+$272.74K</t>
+          <t>+$270.42K</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -5249,32 +5220,36 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>29098.28</v>
+        <v>28482.85</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>29050</v>
+        <v>692</v>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>-$52.34K</t>
+          <t>-$193.19K</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>+$270.42K</t>
+          <t>+$202.70K</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -5283,24 +5258,24 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>28482.85</v>
+        <v>29108.28</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>692</v>
+        <v>29060</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>-$193.19K</t>
+          <t>-$165.74K</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>+$202.70K</t>
+          <t>+$200.63K</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -5310,7 +5285,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5321,24 +5296,24 @@
         </is>
       </c>
       <c r="B59" s="5" t="n">
-        <v>29108.28</v>
+        <v>29118.28</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>29060</v>
+        <v>29070</v>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>-$165.74K</t>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>+$39.25K</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>+$200.63K</t>
+          <t>+$196.27K</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -5348,119 +5323,119 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>29248.28</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>29200</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>+$48.85K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$179.12K</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>29298.28</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>29250</v>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>+$30.24K</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>+$166.32K</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>29028.28</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>28980</v>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>-$130.27K</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>+$130.27K</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>29118.28</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>29070</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>+$39.25K</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>+$196.27K</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="n">
-        <v>29248.28</v>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>29200</v>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>+$48.85K</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>+$179.12K</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="n">
-        <v>29298.28</v>
-      </c>
-      <c r="C62" s="5" t="n">
-        <v>29250</v>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>+$30.24K</t>
-        </is>
-      </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>+$166.32K</t>
-        </is>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -5469,10 +5444,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>29028.28</v>
+        <v>29208.28</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>28980</v>
+        <v>29160</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
@@ -5481,12 +5456,12 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>-$130.27K</t>
+          <t>-$17.45K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$130.27K</t>
+          <t>+$113.40K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -5501,40 +5476,40 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B64" s="2" t="n">
-        <v>29208.28</v>
-      </c>
-      <c r="C64" s="2" t="n">
-        <v>29160</v>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="B64" s="5" t="n">
+        <v>29218.28</v>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>29170</v>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t>-$17.45K</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>+$113.40K</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>+$69.79K</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>+$104.68K</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5545,10 +5520,10 @@
         </is>
       </c>
       <c r="B65" s="5" t="n">
-        <v>29218.28</v>
+        <v>29198.28</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>29170</v>
+        <v>29150</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
@@ -5557,12 +5532,12 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>+$69.79K</t>
+          <t>+$74.15K</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>+$104.68K</t>
+          <t>+$100.32K</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -5577,40 +5552,40 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B66" s="5" t="n">
-        <v>29198.28</v>
-      </c>
-      <c r="C66" s="5" t="n">
-        <v>29150</v>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="B66" s="2" t="n">
+        <v>28948.28</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>28900</v>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>+$74.15K</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>+$100.32K</t>
-        </is>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>-$79.96K</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>+$92.76K</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5621,10 +5596,10 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>28948.28</v>
+        <v>29168.28</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>28900</v>
+        <v>29120</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
@@ -5633,12 +5608,12 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>-$79.96K</t>
+          <t>-$30.53K</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>+$92.76K</t>
+          <t>+$91.59K</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -5659,10 +5634,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>29168.28</v>
+        <v>28973.28</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>29120</v>
+        <v>28925</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
@@ -5671,12 +5646,12 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>-$30.53K</t>
+          <t>-$76.76K</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>+$91.59K</t>
+          <t>+$83.74K</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -5691,38 +5666,38 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B69" s="2" t="n">
-        <v>28973.28</v>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>28925</v>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
+      <c r="B69" s="5" t="n">
+        <v>29228.28</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>29180</v>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-$76.76K</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>+$83.74K</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>-$13.08K</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>+$82.87K</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -5735,24 +5710,24 @@
         </is>
       </c>
       <c r="B70" s="5" t="n">
-        <v>29228.28</v>
+        <v>29068.28</v>
       </c>
       <c r="C70" s="5" t="n">
-        <v>29180</v>
+        <v>29020</v>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr">
-        <is>
-          <t>-$13.08K</t>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>+$4.07K</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>+$82.87K</t>
+          <t>+$77.35K</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
@@ -5762,83 +5737,83 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>29273.28</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>29225</v>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>+$36.64K</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>+$77.35K</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>29268.28</v>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>29220</v>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>+$65.13K</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="n">
-        <v>29068.28</v>
-      </c>
-      <c r="C71" s="5" t="n">
-        <v>29020</v>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>+$4.07K</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>+$77.35K</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n">
-        <v>29273.28</v>
-      </c>
-      <c r="C72" s="2" t="n">
-        <v>29225</v>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E72" s="9" t="inlineStr">
-        <is>
-          <t>+$36.64K</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>+$77.35K</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5849,24 +5824,24 @@
         </is>
       </c>
       <c r="B73" s="5" t="n">
-        <v>29268.28</v>
+        <v>28988.28</v>
       </c>
       <c r="C73" s="5" t="n">
-        <v>29220</v>
+        <v>28940</v>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>$0</t>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>-$24.42K</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>+$65.13K</t>
+          <t>+$24.42K</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -5876,7 +5851,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5887,10 +5862,10 @@
         </is>
       </c>
       <c r="B74" s="5" t="n">
-        <v>28988.28</v>
+        <v>28958.28</v>
       </c>
       <c r="C74" s="5" t="n">
-        <v>28940</v>
+        <v>28910</v>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
@@ -5899,12 +5874,12 @@
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>-$24.42K</t>
+          <t>-$17.45K</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>+$24.42K</t>
+          <t>+$17.45K</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -5918,46 +5893,8 @@
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="n">
-        <v>28958.28</v>
-      </c>
-      <c r="C75" s="5" t="n">
-        <v>28910</v>
-      </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
-        <is>
-          <t>-$17.45K</t>
-        </is>
-      </c>
-      <c r="F75" s="6" t="inlineStr">
-        <is>
-          <t>+$17.45K</t>
-        </is>
-      </c>
-      <c r="G75" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H75"/>
+  <autoFilter ref="A1:H74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>